<commit_message>
Rework Mass Total Services 2025 balance for amended return
Distributions stay at 220,000 (current-year profit only); unrecorded
withdrawals of 119,022 are carried as a loan to the shareholder.
Use EIN 93-3675961 from the accepted return, add the amended-return
explanation statement and corrected Massachusetts schedule values,
and drop the superseded statement PDF.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NFYQ2FQ8VQj9k2seUMu2aV
</commit_message>
<xml_diff>
--- a/mass-total-services-2025/MassTotalServices_2025_Balance_L_M1_M2.xlsx
+++ b/mass-total-services-2025/MassTotalServices_2025_Balance_L_M1_M2.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -495,143 +495,125 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CORRECOES (o que muda na declaracao federal):</t>
+          <t>DECLARACAO RETIFICADORA (1120-S 2025, EIN 93-3675961) - o que muda:</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>1. Distribuicoes K 16d e K-1 16D: 220,000 -&gt; 339,022. Retiradas do socio sem nota promissoria/juros = distribuicao (IRC 1368).</t>
+          <t>1. Pagina 1, item F (Total assets): 7,909 -&gt; 126,931.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2. Schedule M-2: linha 7 = 307,412 (limitada ao AAA) e linha 8 = 0. O excesso de 31,610 nao entra no M-2.</t>
+          <t>2. Schedule L inicio: caixa 77,714 e retained earnings 77,714 (estava tudo zero).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>3. Schedule L inicio: estava zerado; deve ser o saldo final de 2024 (caixa e lucros acumulados 77,714).</t>
+          <t>3. Schedule L fim: Loans to shareholders (L7) 119,022; financiamento do BMW sai da L16 e vai para a L20; retained earnings 87,412.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>4. Schedule L fim: Retained earnings (31,610) (igual ao original). O 39,519 sai de Accounts payable (L16) e vai para notes payable (L20).</t>
+          <t>4. Schedule M-1, M-2, Schedule K e K-1: sem alteracao (distribuicoes 220,000; AAA final 87,412).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>5. Socio: distribuicao excede a base em 31,610 = ganho de capital de longo prazo no 1040 (Form 8949/Sch D). Form 7203 obrigatorio.</t>
+          <t>5. Form 4562: BMW na Part V (listed property). K-1: tirar 'PRESIDENT' do nome do socio.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>6. Form 4562: o BMW estava na Part II (nao listado). Carro e listed property -&gt; Part V, com % de uso e milhas (Section B).</t>
+          <t>6. Massachusetts: Schedules A, B e D com os novos saldos; excise continua 456.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>7. K-1: o nome do socio esta 'ERLI MARQUES DE MORAIS PRESIDENT' - remover 'PRESIDENT' do campo de nome.</t>
-        </is>
-      </c>
+      <c r="A12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>PARA O EMPRESTIMO AO SOCIO SER ACEITO PELO IRS:</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>PENDENCIAS (mudam os numeros - ajustar na aba Dados):</t>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>a. Nota promissoria assinada (valor 119,022, juros pela taxa AFR do IRS, prazo de pagamento).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>a. Modelo do BMW: se for carro de passeio ate 6,000 lbs, a depreciacao fica limitada a 20,200 (IRC 280F). Mudar Dados!B13 para 1.</t>
+          <t>b. Cobrar juros pela AFR - sem juros, o IRS imputa juros (IRC 7872).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>b. Log de milhas: uso comercial precisa ser &gt; 50% para ter bonus; % menor reduz a depreciacao (Dados!B12).</t>
+          <t>c. O socio precisa devolver de fato (pagamentos registrados no banco).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>c. Extrato 31/12/2024: se o caixa era menor que 77,714, a diferenca foi retirada em 2024 -&gt; emendar K-1 2024 (16D).</t>
+          <t>d. Sem isso, o IRS pode tratar os 119,022 como distribuicao (mude Dados!B22 para 0 para ver o efeito).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>d. Contrato do financiamento: saldo em 31/12/2025 e juros pagos (dedutiveis na linha 13).</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>e. Capital aportado pelo socio na abertura (2023): aumenta a base e reduz o ganho de capital (Dados!B21).</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRMAR:</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>f. Gifts 1,671: so $25 por pessoa por ano e dedutivel (IRC 274(b)); excesso em Dados!B20.</t>
+          <t>e. Extrato de 31/12/2024 (caixa inicial 77,714 reconstruido). Diferenca vai para Loans to shareholders no inicio.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>g. Salario do socio: S corp com socio que trabalha precisa pagar salario razoavel via payroll (W-2). Iniciar em 2026.</t>
+          <t>f. Modelo/GVWR do BMW e log de milhas (Dados!B12 e B13).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>h. 1099: Schedule B Q14 em branco - se pagou terceirizados &gt;= $600 (incluido nas compras de 128,185), emitir 1099-NEC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>i. Prazo: 1120-S com extensao vencia 15/09/2026. Se ainda nao foi transmitida, transmitir ja; multa $255/socio/mes (pedir First-Time Abatement).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>j. Massachusetts: o balanco final e o mesmo ja declarado no Schedule A (caixa 7,909, passivo 39,519, capital -31,610).</t>
+          <t>g. Contrato do financiamento: saldo em 31/12/2025 e juros pagos.</t>
         </is>
       </c>
     </row>
@@ -646,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="66" customWidth="1" min="1" max="1"/>
@@ -666,7 +648,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>
@@ -927,13 +909,28 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Retiradas do socio sem registro: 1 = emprestimo ao socio, 0 = distribuicao</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Distribuicoes de 2025 foram so 220,000 -&gt; emprestimo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Depreciacao calculada (federal)</t>
         </is>
       </c>
-      <c r="B23" s="10">
+      <c r="B24" s="10">
         <f>IF(Dados!$B$13=1,MIN(Dados!$B$11*Dados!$B$12,Dados!$B$14),Dados!$B$11*Dados!$B$12)</f>
         <v/>
       </c>
@@ -969,7 +966,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1044,7 @@
         </is>
       </c>
       <c r="B11" s="11">
-        <f>-Dados!$B$23</f>
+        <f>-Dados!$B$24</f>
         <v/>
       </c>
     </row>
@@ -1106,7 +1103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1126,7 +1123,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1175,7 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>Dados!$B$23</f>
+        <f>Dados!$B$24</f>
         <v/>
       </c>
     </row>
@@ -1240,7 +1237,7 @@
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Retiradas nao registradas (distribuicao adicional)</t>
+          <t>Retiradas do socio nao registradas</t>
         </is>
       </c>
       <c r="B14" s="15">
@@ -1255,7 +1252,18 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>Dados!$B$15+B14</f>
+        <f>Dados!$B$15+IF(Dados!$B$22=1,0,B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Emprestimo ao socio (Sch L linha 7)</t>
+        </is>
+      </c>
+      <c r="B17" s="12">
+        <f>IF(Dados!$B$22=1,B14,0)</f>
         <v/>
       </c>
     </row>
@@ -1290,7 +1298,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>
@@ -1346,36 +1354,50 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>10a Buildings and other depreciable assets (BMW)</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="n">
+          <t>7  Loans to shareholders</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="11">
-        <f>Dados!$B$11</f>
+      <c r="E7" s="11">
+        <f>Conciliacao!B17</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>10b Less accumulated depreciation  (liquido em b/d)</t>
+          <t>10a Buildings and other depreciable assets (BMW)</t>
         </is>
       </c>
       <c r="B8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="11">
-        <f>B7+B8</f>
-        <v/>
-      </c>
       <c r="D8" s="11">
-        <f>-Dados!$B$23</f>
-        <v/>
-      </c>
-      <c r="E8" s="11">
-        <f>D7+D8</f>
+        <f>Dados!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>10b Less accumulated depreciation  (liquido em b/d)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="11">
+        <f>B8+B9</f>
+        <v/>
+      </c>
+      <c r="D9" s="11">
+        <f>-Dados!$B$24</f>
+        <v/>
+      </c>
+      <c r="E9" s="11">
+        <f>D8+D9</f>
         <v/>
       </c>
     </row>
@@ -1386,11 +1408,11 @@
         </is>
       </c>
       <c r="C10" s="12">
-        <f>C6+C8</f>
+        <f>C6+C7+C9</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>E6+E8</f>
+        <f>E6+E7+E9</f>
         <v/>
       </c>
     </row>
@@ -1499,7 +1521,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1653,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1840,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mass Total Services Inc  -  EIN 93-3675960  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
+          <t>Mass Total Services Inc  -  EIN 93-3675961  -  Form 1120-S 2025 (ano-calendario, regime de caixa)</t>
         </is>
       </c>
     </row>

</xml_diff>